<commit_message>
chore: ignore generated graphify artifacts and sync project updates
</commit_message>
<xml_diff>
--- a/src/data/Color Guide.xlsx
+++ b/src/data/Color Guide.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\programming\viomes\homepage\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\MARKETING\1. PRODUCT\Χρώματα\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3BA34CAD-BD95-499D-9014-D670B23E746B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0393E4A2-EA58-462B-8A2C-03249D8BF903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B6F5591D-9278-43FC-8DF2-ACFCB49B508B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6F5591D-9278-43FC-8DF2-ACFCB49B508B}"/>
   </bookViews>
   <sheets>
     <sheet name="Φύλλο1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Φύλλο1!$B$1:$G$105</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="500">
   <si>
     <t>Viomes Color</t>
   </si>
@@ -1440,6 +1443,102 @@
   </si>
   <si>
     <t>#1B282D</t>
+  </si>
+  <si>
+    <t>Petrol</t>
+  </si>
+  <si>
+    <t>Mustard</t>
+  </si>
+  <si>
+    <t>Aubergine</t>
+  </si>
+  <si>
+    <t>Moss</t>
+  </si>
+  <si>
+    <t>Indigo</t>
+  </si>
+  <si>
+    <t>Cloud</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baby blue </t>
+  </si>
+  <si>
+    <t>Πετρόλ</t>
+  </si>
+  <si>
+    <t>Μουσταρδί</t>
+  </si>
+  <si>
+    <t>Μελιτζανί</t>
+  </si>
+  <si>
+    <t>Πράσινο Μος</t>
+  </si>
+  <si>
+    <t>Ίντιγκο</t>
+  </si>
+  <si>
+    <t>Σύννεφο</t>
+  </si>
+  <si>
+    <t>Σκούρο Σιέλ</t>
+  </si>
+  <si>
+    <t>60-85-35-35</t>
+  </si>
+  <si>
+    <t>511 C</t>
+  </si>
+  <si>
+    <t>20-40-100-8</t>
+  </si>
+  <si>
+    <t>1245 C</t>
+  </si>
+  <si>
+    <t>55-35-73-23</t>
+  </si>
+  <si>
+    <t>5763 C</t>
+  </si>
+  <si>
+    <t>100-100-37-30</t>
+  </si>
+  <si>
+    <t>47-36-34-15</t>
+  </si>
+  <si>
+    <t>Cool Gray 8 C</t>
+  </si>
+  <si>
+    <t>100-58-45-47</t>
+  </si>
+  <si>
+    <t>548 C</t>
+  </si>
+  <si>
+    <t>56-30-24-6</t>
+  </si>
+  <si>
+    <t>#003D4C</t>
+  </si>
+  <si>
+    <t>#C69214</t>
+  </si>
+  <si>
+    <t>#612C51</t>
+  </si>
+  <si>
+    <t>#737B4C</t>
+  </si>
+  <si>
+    <t>#000070</t>
+  </si>
+  <si>
+    <t>#69a8b6</t>
   </si>
 </sst>
 </file>
@@ -1506,7 +1605,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Κανονικό" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1838,7 +1937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA5DDEC7-DAB3-47BC-BD0A-41C4E2DEB58D}">
-  <dimension ref="B1:G105"/>
+  <dimension ref="B1:G112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.140625" style="1" customWidth="1"/>
@@ -3703,7 +3802,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="97" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B97" s="1">
         <v>97</v>
       </c>
@@ -3714,7 +3813,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="98" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B98" s="1">
         <v>98</v>
       </c>
@@ -3725,7 +3824,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="99" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B99" s="1">
         <v>200</v>
       </c>
@@ -3733,7 +3832,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="100" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B100" s="1">
         <v>300</v>
       </c>
@@ -3741,7 +3840,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="101" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B101" s="1">
         <v>310</v>
       </c>
@@ -3749,7 +3848,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="102" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B102" s="1">
         <v>320</v>
       </c>
@@ -3757,7 +3856,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="103" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B103" s="1">
         <v>330</v>
       </c>
@@ -3765,7 +3864,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="104" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B104" s="1">
         <v>340</v>
       </c>
@@ -3773,7 +3872,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="105" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B105" s="1">
         <v>350</v>
       </c>
@@ -3781,7 +3880,145 @@
         <v>384</v>
       </c>
     </row>
+    <row r="106" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B106" s="1">
+        <v>138</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="107" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B107" s="1">
+        <v>189</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="108" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B108" s="1">
+        <v>111</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B109" s="1">
+        <v>184</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="110" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B110" s="1">
+        <v>139</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="111" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B111" s="1">
+        <v>163</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="112" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B112" s="1">
+        <v>173</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>499</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="B1:G105" xr:uid="{CA5DDEC7-DAB3-47BC-BD0A-41C4E2DEB58D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>